<commit_message>
MB001 #364: atomic correction candidate
</commit_message>
<xml_diff>
--- a/products-storage/07-uderzhaniya-shtrafy-zachety/04-raschet-ubytkov.xlsx
+++ b/products-storage/07-uderzhaniya-shtrafy-zachety/04-raschet-ubytkov.xlsx
@@ -89,7 +89,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -110,6 +110,7 @@
     </xf>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="49" fontId="0" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="49" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -499,10 +500,10 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="76" customHeight="1">
+    <row r="2" ht="106" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Вводите данные только в жёлтые ячейки. Суммы — в рублях. Ставка — числом процентов: 0,05 % в день вводится как 0,05, 16 % годовых — как 16, без знака %: с ним Calc и Excel хранят 0,05 % как 0,0005. Поэтому ставка пеней меньше 0,01 % в день и ключевая ставка меньше 1 % годовых не считаются — в «Проверке» будет сообщение. Даты — ДД.ММ.ГГГГ; первый и последний день периода входят в число дней. Период с другой базой или ставкой — отдельной строкой. Если в столбце «Проверка» есть сообщение, сумма по этой строке и итог раздела не считаются.</t>
+          <t>Вводите данные только в жёлтые ячейки. Суммы — в рублях. Ставку в таблицах пеней и ст. 395 набирайте с клавиатуры: ячейка текстовая, 0,05 и 0,05% — это 0,05 % в день, 16 и 16% — 16 % годовых. Если в ячейке ставки число (вставка из другой таблицы, формула), знак % по нему не виден — строка не считается; наберите ставку заново с апострофом впереди: '0,05. Ставка пеней меньше 0,01 % в день и ключевая ставка меньше 1 % годовых не считаются. Процент штрафа в п. 2.2 — числом без знака %: 5 % — как 5. Даты — ДД.ММ.ГГГГ; первый и последний день периода входят в число дней. Период с другой базой или ставкой — отдельной строкой. Если в столбце «Проверка» есть сообщение, сумма по этой строке и итог раздела не считаются.</t>
         </is>
       </c>
     </row>
@@ -652,7 +653,7 @@
       </c>
       <c r="F17" s="9" t="inlineStr">
         <is>
-          <t>Ставка, % в день (без знака %)</t>
+          <t>Ставка, % в день (0,05 или 0,05%)</t>
         </is>
       </c>
       <c r="G17" s="9" t="inlineStr">
@@ -677,13 +678,13 @@
         <v/>
       </c>
       <c r="E18" s="5" t="n"/>
-      <c r="F18" s="8" t="n"/>
-      <c r="G18" s="12">
-        <f>IF(OR(H18&lt;&gt;"",B18=""),"",E18*F18/100*D18)</f>
-        <v/>
-      </c>
-      <c r="H18" s="13">
-        <f>IF(AND(B18="",C18="",E18="",F18=""),"",IF(OR(B18="",C18="",E18="",F18=""),"Заполните все поля строки: начало, окончание, базу и ставку",IF(OR(NOT(ISNUMBER(B18)),NOT(ISNUMBER(C18)),NOT(ISNUMBER(E18)),NOT(ISNUMBER(F18))),"Даты и суммы вводятся числом, даты — ДД.ММ.ГГГГ",IF(C18&lt;B18,"Окончание раньше начала — проверьте даты",IF(OR(E18&lt;0,F18&lt;0),"База или ставка меньше нуля — проверьте ввод",IF(AND(F18&gt;0,F18&lt;0.01),"Ставка меньше 0,01 % в день — так бывает, если набрать знак %. Введите число без знака %: 0,05 % — как 0,05",""))))))</f>
+      <c r="F18" s="12" t="n"/>
+      <c r="G18" s="13">
+        <f>IF(OR(H18&lt;&gt;"",B18=""),"",E18*_xlfn.NUMBERVALUE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F18," ",""),"%",""),"'",""),".",","),","," ")/100*D18)</f>
+        <v/>
+      </c>
+      <c r="H18" s="14">
+        <f>IF(AND(B18="",C18="",E18="",F18=""),"",IF(OR(B18="",C18="",E18="",F18=""),"Заполните все поля строки: начало, окончание, базу и ставку",IF(OR(NOT(ISNUMBER(B18)),NOT(ISNUMBER(C18)),NOT(ISNUMBER(E18))),"Даты и суммы вводятся числом, даты — ДД.ММ.ГГГГ",IF(ISNUMBER(F18),"Ставка вставлена числом — не видно, был ли знак %. Наберите её заново с апострофом впереди: '0,1 или '0,1%",IF(OR(NOT(ISTEXT(F18)),SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F18," ",""),"%",""),"'",""),".",",")="",ISERROR(_xlfn.NUMBERVALUE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F18," ",""),"%",""),"'",""),".",","),","," "))),"Ставка не распознана — наберите число, например 0,1 или 0,1%",IF(C18&lt;B18,"Окончание раньше начала — проверьте даты",IF(OR(E18&lt;0,_xlfn.NUMBERVALUE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F18," ",""),"%",""),"'",""),".",","),","," ")&lt;0),"База или ставка меньше нуля — проверьте ввод",IF(AND(_xlfn.NUMBERVALUE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F18," ",""),"%",""),"'",""),".",","),","," ")&gt;0,_xlfn.NUMBERVALUE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F18," ",""),"%",""),"'",""),".",","),","," ")&lt;0.01),"Ставка меньше 0,01 % в день — книга такую ставку не считает",""))))))))</f>
         <v/>
       </c>
     </row>
@@ -698,13 +699,13 @@
         <v/>
       </c>
       <c r="E19" s="5" t="n"/>
-      <c r="F19" s="8" t="n"/>
-      <c r="G19" s="12">
-        <f>IF(OR(H19&lt;&gt;"",B19=""),"",E19*F19/100*D19)</f>
-        <v/>
-      </c>
-      <c r="H19" s="13">
-        <f>IF(AND(B19="",C19="",E19="",F19=""),"",IF(OR(B19="",C19="",E19="",F19=""),"Заполните все поля строки: начало, окончание, базу и ставку",IF(OR(NOT(ISNUMBER(B19)),NOT(ISNUMBER(C19)),NOT(ISNUMBER(E19)),NOT(ISNUMBER(F19))),"Даты и суммы вводятся числом, даты — ДД.ММ.ГГГГ",IF(C19&lt;B19,"Окончание раньше начала — проверьте даты",IF(OR(E19&lt;0,F19&lt;0),"База или ставка меньше нуля — проверьте ввод",IF(AND(F19&gt;0,F19&lt;0.01),"Ставка меньше 0,01 % в день — так бывает, если набрать знак %. Введите число без знака %: 0,05 % — как 0,05",""))))))</f>
+      <c r="F19" s="12" t="n"/>
+      <c r="G19" s="13">
+        <f>IF(OR(H19&lt;&gt;"",B19=""),"",E19*_xlfn.NUMBERVALUE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F19," ",""),"%",""),"'",""),".",","),","," ")/100*D19)</f>
+        <v/>
+      </c>
+      <c r="H19" s="14">
+        <f>IF(AND(B19="",C19="",E19="",F19=""),"",IF(OR(B19="",C19="",E19="",F19=""),"Заполните все поля строки: начало, окончание, базу и ставку",IF(OR(NOT(ISNUMBER(B19)),NOT(ISNUMBER(C19)),NOT(ISNUMBER(E19))),"Даты и суммы вводятся числом, даты — ДД.ММ.ГГГГ",IF(ISNUMBER(F19),"Ставка вставлена числом — не видно, был ли знак %. Наберите её заново с апострофом впереди: '0,1 или '0,1%",IF(OR(NOT(ISTEXT(F19)),SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F19," ",""),"%",""),"'",""),".",",")="",ISERROR(_xlfn.NUMBERVALUE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F19," ",""),"%",""),"'",""),".",","),","," "))),"Ставка не распознана — наберите число, например 0,1 или 0,1%",IF(C19&lt;B19,"Окончание раньше начала — проверьте даты",IF(OR(E19&lt;0,_xlfn.NUMBERVALUE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F19," ",""),"%",""),"'",""),".",","),","," ")&lt;0),"База или ставка меньше нуля — проверьте ввод",IF(AND(_xlfn.NUMBERVALUE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F19," ",""),"%",""),"'",""),".",","),","," ")&gt;0,_xlfn.NUMBERVALUE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F19," ",""),"%",""),"'",""),".",","),","," ")&lt;0.01),"Ставка меньше 0,01 % в день — книга такую ставку не считает",""))))))))</f>
         <v/>
       </c>
     </row>
@@ -719,13 +720,13 @@
         <v/>
       </c>
       <c r="E20" s="5" t="n"/>
-      <c r="F20" s="8" t="n"/>
-      <c r="G20" s="12">
-        <f>IF(OR(H20&lt;&gt;"",B20=""),"",E20*F20/100*D20)</f>
-        <v/>
-      </c>
-      <c r="H20" s="13">
-        <f>IF(AND(B20="",C20="",E20="",F20=""),"",IF(OR(B20="",C20="",E20="",F20=""),"Заполните все поля строки: начало, окончание, базу и ставку",IF(OR(NOT(ISNUMBER(B20)),NOT(ISNUMBER(C20)),NOT(ISNUMBER(E20)),NOT(ISNUMBER(F20))),"Даты и суммы вводятся числом, даты — ДД.ММ.ГГГГ",IF(C20&lt;B20,"Окончание раньше начала — проверьте даты",IF(OR(E20&lt;0,F20&lt;0),"База или ставка меньше нуля — проверьте ввод",IF(AND(F20&gt;0,F20&lt;0.01),"Ставка меньше 0,01 % в день — так бывает, если набрать знак %. Введите число без знака %: 0,05 % — как 0,05",""))))))</f>
+      <c r="F20" s="12" t="n"/>
+      <c r="G20" s="13">
+        <f>IF(OR(H20&lt;&gt;"",B20=""),"",E20*_xlfn.NUMBERVALUE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F20," ",""),"%",""),"'",""),".",","),","," ")/100*D20)</f>
+        <v/>
+      </c>
+      <c r="H20" s="14">
+        <f>IF(AND(B20="",C20="",E20="",F20=""),"",IF(OR(B20="",C20="",E20="",F20=""),"Заполните все поля строки: начало, окончание, базу и ставку",IF(OR(NOT(ISNUMBER(B20)),NOT(ISNUMBER(C20)),NOT(ISNUMBER(E20))),"Даты и суммы вводятся числом, даты — ДД.ММ.ГГГГ",IF(ISNUMBER(F20),"Ставка вставлена числом — не видно, был ли знак %. Наберите её заново с апострофом впереди: '0,1 или '0,1%",IF(OR(NOT(ISTEXT(F20)),SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F20," ",""),"%",""),"'",""),".",",")="",ISERROR(_xlfn.NUMBERVALUE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F20," ",""),"%",""),"'",""),".",","),","," "))),"Ставка не распознана — наберите число, например 0,1 или 0,1%",IF(C20&lt;B20,"Окончание раньше начала — проверьте даты",IF(OR(E20&lt;0,_xlfn.NUMBERVALUE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F20," ",""),"%",""),"'",""),".",","),","," ")&lt;0),"База или ставка меньше нуля — проверьте ввод",IF(AND(_xlfn.NUMBERVALUE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F20," ",""),"%",""),"'",""),".",","),","," ")&gt;0,_xlfn.NUMBERVALUE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F20," ",""),"%",""),"'",""),".",","),","," ")&lt;0.01),"Ставка меньше 0,01 % в день — книга такую ставку не считает",""))))))))</f>
         <v/>
       </c>
     </row>
@@ -740,13 +741,13 @@
         <v/>
       </c>
       <c r="E21" s="5" t="n"/>
-      <c r="F21" s="8" t="n"/>
-      <c r="G21" s="12">
-        <f>IF(OR(H21&lt;&gt;"",B21=""),"",E21*F21/100*D21)</f>
-        <v/>
-      </c>
-      <c r="H21" s="13">
-        <f>IF(AND(B21="",C21="",E21="",F21=""),"",IF(OR(B21="",C21="",E21="",F21=""),"Заполните все поля строки: начало, окончание, базу и ставку",IF(OR(NOT(ISNUMBER(B21)),NOT(ISNUMBER(C21)),NOT(ISNUMBER(E21)),NOT(ISNUMBER(F21))),"Даты и суммы вводятся числом, даты — ДД.ММ.ГГГГ",IF(C21&lt;B21,"Окончание раньше начала — проверьте даты",IF(OR(E21&lt;0,F21&lt;0),"База или ставка меньше нуля — проверьте ввод",IF(AND(F21&gt;0,F21&lt;0.01),"Ставка меньше 0,01 % в день — так бывает, если набрать знак %. Введите число без знака %: 0,05 % — как 0,05",""))))))</f>
+      <c r="F21" s="12" t="n"/>
+      <c r="G21" s="13">
+        <f>IF(OR(H21&lt;&gt;"",B21=""),"",E21*_xlfn.NUMBERVALUE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F21," ",""),"%",""),"'",""),".",","),","," ")/100*D21)</f>
+        <v/>
+      </c>
+      <c r="H21" s="14">
+        <f>IF(AND(B21="",C21="",E21="",F21=""),"",IF(OR(B21="",C21="",E21="",F21=""),"Заполните все поля строки: начало, окончание, базу и ставку",IF(OR(NOT(ISNUMBER(B21)),NOT(ISNUMBER(C21)),NOT(ISNUMBER(E21))),"Даты и суммы вводятся числом, даты — ДД.ММ.ГГГГ",IF(ISNUMBER(F21),"Ставка вставлена числом — не видно, был ли знак %. Наберите её заново с апострофом впереди: '0,1 или '0,1%",IF(OR(NOT(ISTEXT(F21)),SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F21," ",""),"%",""),"'",""),".",",")="",ISERROR(_xlfn.NUMBERVALUE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F21," ",""),"%",""),"'",""),".",","),","," "))),"Ставка не распознана — наберите число, например 0,1 или 0,1%",IF(C21&lt;B21,"Окончание раньше начала — проверьте даты",IF(OR(E21&lt;0,_xlfn.NUMBERVALUE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F21," ",""),"%",""),"'",""),".",","),","," ")&lt;0),"База или ставка меньше нуля — проверьте ввод",IF(AND(_xlfn.NUMBERVALUE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F21," ",""),"%",""),"'",""),".",","),","," ")&gt;0,_xlfn.NUMBERVALUE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F21," ",""),"%",""),"'",""),".",","),","," ")&lt;0.01),"Ставка меньше 0,01 % в день — книга такую ставку не считает",""))))))))</f>
         <v/>
       </c>
     </row>
@@ -761,13 +762,13 @@
         <v/>
       </c>
       <c r="E22" s="5" t="n"/>
-      <c r="F22" s="8" t="n"/>
-      <c r="G22" s="12">
-        <f>IF(OR(H22&lt;&gt;"",B22=""),"",E22*F22/100*D22)</f>
-        <v/>
-      </c>
-      <c r="H22" s="13">
-        <f>IF(AND(B22="",C22="",E22="",F22=""),"",IF(OR(B22="",C22="",E22="",F22=""),"Заполните все поля строки: начало, окончание, базу и ставку",IF(OR(NOT(ISNUMBER(B22)),NOT(ISNUMBER(C22)),NOT(ISNUMBER(E22)),NOT(ISNUMBER(F22))),"Даты и суммы вводятся числом, даты — ДД.ММ.ГГГГ",IF(C22&lt;B22,"Окончание раньше начала — проверьте даты",IF(OR(E22&lt;0,F22&lt;0),"База или ставка меньше нуля — проверьте ввод",IF(AND(F22&gt;0,F22&lt;0.01),"Ставка меньше 0,01 % в день — так бывает, если набрать знак %. Введите число без знака %: 0,05 % — как 0,05",""))))))</f>
+      <c r="F22" s="12" t="n"/>
+      <c r="G22" s="13">
+        <f>IF(OR(H22&lt;&gt;"",B22=""),"",E22*_xlfn.NUMBERVALUE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F22," ",""),"%",""),"'",""),".",","),","," ")/100*D22)</f>
+        <v/>
+      </c>
+      <c r="H22" s="14">
+        <f>IF(AND(B22="",C22="",E22="",F22=""),"",IF(OR(B22="",C22="",E22="",F22=""),"Заполните все поля строки: начало, окончание, базу и ставку",IF(OR(NOT(ISNUMBER(B22)),NOT(ISNUMBER(C22)),NOT(ISNUMBER(E22))),"Даты и суммы вводятся числом, даты — ДД.ММ.ГГГГ",IF(ISNUMBER(F22),"Ставка вставлена числом — не видно, был ли знак %. Наберите её заново с апострофом впереди: '0,1 или '0,1%",IF(OR(NOT(ISTEXT(F22)),SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F22," ",""),"%",""),"'",""),".",",")="",ISERROR(_xlfn.NUMBERVALUE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F22," ",""),"%",""),"'",""),".",","),","," "))),"Ставка не распознана — наберите число, например 0,1 или 0,1%",IF(C22&lt;B22,"Окончание раньше начала — проверьте даты",IF(OR(E22&lt;0,_xlfn.NUMBERVALUE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F22," ",""),"%",""),"'",""),".",","),","," ")&lt;0),"База или ставка меньше нуля — проверьте ввод",IF(AND(_xlfn.NUMBERVALUE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F22," ",""),"%",""),"'",""),".",","),","," ")&gt;0,_xlfn.NUMBERVALUE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F22," ",""),"%",""),"'",""),".",","),","," ")&lt;0.01),"Ставка меньше 0,01 % в день — книга такую ставку не считает",""))))))))</f>
         <v/>
       </c>
     </row>
@@ -821,7 +822,7 @@
       </c>
       <c r="F26" s="9" t="inlineStr">
         <is>
-          <t>Ключевая ставка, % годовых (без знака %)</t>
+          <t>Ключевая ставка, % годовых (16 или 16%)</t>
         </is>
       </c>
       <c r="G26" s="9" t="inlineStr">
@@ -846,13 +847,13 @@
         <v/>
       </c>
       <c r="E27" s="5" t="n"/>
-      <c r="F27" s="8" t="n"/>
-      <c r="G27" s="12">
-        <f>IF(OR(H27&lt;&gt;"",B27=""),"",E27*F27/100/365*D27)</f>
-        <v/>
-      </c>
-      <c r="H27" s="13">
-        <f>IF(AND(B27="",C27="",E27="",F27=""),"",IF(OR(B27="",C27="",E27="",F27=""),"Заполните все поля строки: начало, окончание, базу и ставку",IF(OR(NOT(ISNUMBER(B27)),NOT(ISNUMBER(C27)),NOT(ISNUMBER(E27)),NOT(ISNUMBER(F27))),"Даты и суммы вводятся числом, даты — ДД.ММ.ГГГГ",IF(C27&lt;B27,"Окончание раньше начала — проверьте даты",IF(OR(E27&lt;0,F27&lt;0),"База или ставка меньше нуля — проверьте ввод",IF(AND(F27&gt;0,F27&lt;1),"Ставка меньше 1 % годовых — так бывает, если набрать знак %. Введите число без знака %: 16 % — как 16",""))))))</f>
+      <c r="F27" s="12" t="n"/>
+      <c r="G27" s="13">
+        <f>IF(OR(H27&lt;&gt;"",B27=""),"",E27*_xlfn.NUMBERVALUE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F27," ",""),"%",""),"'",""),".",","),","," ")/100/365*D27)</f>
+        <v/>
+      </c>
+      <c r="H27" s="14">
+        <f>IF(AND(B27="",C27="",E27="",F27=""),"",IF(OR(B27="",C27="",E27="",F27=""),"Заполните все поля строки: начало, окончание, базу и ставку",IF(OR(NOT(ISNUMBER(B27)),NOT(ISNUMBER(C27)),NOT(ISNUMBER(E27))),"Даты и суммы вводятся числом, даты — ДД.ММ.ГГГГ",IF(ISNUMBER(F27),"Ставка вставлена числом — не видно, был ли знак %. Наберите её заново с апострофом впереди: '0,1 или '0,1%",IF(OR(NOT(ISTEXT(F27)),SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F27," ",""),"%",""),"'",""),".",",")="",ISERROR(_xlfn.NUMBERVALUE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F27," ",""),"%",""),"'",""),".",","),","," "))),"Ставка не распознана — наберите число, например 0,1 или 0,1%",IF(C27&lt;B27,"Окончание раньше начала — проверьте даты",IF(OR(E27&lt;0,_xlfn.NUMBERVALUE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F27," ",""),"%",""),"'",""),".",","),","," ")&lt;0),"База или ставка меньше нуля — проверьте ввод",IF(AND(_xlfn.NUMBERVALUE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F27," ",""),"%",""),"'",""),".",","),","," ")&gt;0,_xlfn.NUMBERVALUE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F27," ",""),"%",""),"'",""),".",","),","," ")&lt;1),"Ставка меньше 1 % годовых — книга такую ставку не считает",""))))))))</f>
         <v/>
       </c>
     </row>
@@ -867,13 +868,13 @@
         <v/>
       </c>
       <c r="E28" s="5" t="n"/>
-      <c r="F28" s="8" t="n"/>
-      <c r="G28" s="12">
-        <f>IF(OR(H28&lt;&gt;"",B28=""),"",E28*F28/100/365*D28)</f>
-        <v/>
-      </c>
-      <c r="H28" s="13">
-        <f>IF(AND(B28="",C28="",E28="",F28=""),"",IF(OR(B28="",C28="",E28="",F28=""),"Заполните все поля строки: начало, окончание, базу и ставку",IF(OR(NOT(ISNUMBER(B28)),NOT(ISNUMBER(C28)),NOT(ISNUMBER(E28)),NOT(ISNUMBER(F28))),"Даты и суммы вводятся числом, даты — ДД.ММ.ГГГГ",IF(C28&lt;B28,"Окончание раньше начала — проверьте даты",IF(OR(E28&lt;0,F28&lt;0),"База или ставка меньше нуля — проверьте ввод",IF(AND(F28&gt;0,F28&lt;1),"Ставка меньше 1 % годовых — так бывает, если набрать знак %. Введите число без знака %: 16 % — как 16",""))))))</f>
+      <c r="F28" s="12" t="n"/>
+      <c r="G28" s="13">
+        <f>IF(OR(H28&lt;&gt;"",B28=""),"",E28*_xlfn.NUMBERVALUE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F28," ",""),"%",""),"'",""),".",","),","," ")/100/365*D28)</f>
+        <v/>
+      </c>
+      <c r="H28" s="14">
+        <f>IF(AND(B28="",C28="",E28="",F28=""),"",IF(OR(B28="",C28="",E28="",F28=""),"Заполните все поля строки: начало, окончание, базу и ставку",IF(OR(NOT(ISNUMBER(B28)),NOT(ISNUMBER(C28)),NOT(ISNUMBER(E28))),"Даты и суммы вводятся числом, даты — ДД.ММ.ГГГГ",IF(ISNUMBER(F28),"Ставка вставлена числом — не видно, был ли знак %. Наберите её заново с апострофом впереди: '0,1 или '0,1%",IF(OR(NOT(ISTEXT(F28)),SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F28," ",""),"%",""),"'",""),".",",")="",ISERROR(_xlfn.NUMBERVALUE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F28," ",""),"%",""),"'",""),".",","),","," "))),"Ставка не распознана — наберите число, например 0,1 или 0,1%",IF(C28&lt;B28,"Окончание раньше начала — проверьте даты",IF(OR(E28&lt;0,_xlfn.NUMBERVALUE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F28," ",""),"%",""),"'",""),".",","),","," ")&lt;0),"База или ставка меньше нуля — проверьте ввод",IF(AND(_xlfn.NUMBERVALUE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F28," ",""),"%",""),"'",""),".",","),","," ")&gt;0,_xlfn.NUMBERVALUE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F28," ",""),"%",""),"'",""),".",","),","," ")&lt;1),"Ставка меньше 1 % годовых — книга такую ставку не считает",""))))))))</f>
         <v/>
       </c>
     </row>
@@ -888,13 +889,13 @@
         <v/>
       </c>
       <c r="E29" s="5" t="n"/>
-      <c r="F29" s="8" t="n"/>
-      <c r="G29" s="12">
-        <f>IF(OR(H29&lt;&gt;"",B29=""),"",E29*F29/100/365*D29)</f>
-        <v/>
-      </c>
-      <c r="H29" s="13">
-        <f>IF(AND(B29="",C29="",E29="",F29=""),"",IF(OR(B29="",C29="",E29="",F29=""),"Заполните все поля строки: начало, окончание, базу и ставку",IF(OR(NOT(ISNUMBER(B29)),NOT(ISNUMBER(C29)),NOT(ISNUMBER(E29)),NOT(ISNUMBER(F29))),"Даты и суммы вводятся числом, даты — ДД.ММ.ГГГГ",IF(C29&lt;B29,"Окончание раньше начала — проверьте даты",IF(OR(E29&lt;0,F29&lt;0),"База или ставка меньше нуля — проверьте ввод",IF(AND(F29&gt;0,F29&lt;1),"Ставка меньше 1 % годовых — так бывает, если набрать знак %. Введите число без знака %: 16 % — как 16",""))))))</f>
+      <c r="F29" s="12" t="n"/>
+      <c r="G29" s="13">
+        <f>IF(OR(H29&lt;&gt;"",B29=""),"",E29*_xlfn.NUMBERVALUE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F29," ",""),"%",""),"'",""),".",","),","," ")/100/365*D29)</f>
+        <v/>
+      </c>
+      <c r="H29" s="14">
+        <f>IF(AND(B29="",C29="",E29="",F29=""),"",IF(OR(B29="",C29="",E29="",F29=""),"Заполните все поля строки: начало, окончание, базу и ставку",IF(OR(NOT(ISNUMBER(B29)),NOT(ISNUMBER(C29)),NOT(ISNUMBER(E29))),"Даты и суммы вводятся числом, даты — ДД.ММ.ГГГГ",IF(ISNUMBER(F29),"Ставка вставлена числом — не видно, был ли знак %. Наберите её заново с апострофом впереди: '0,1 или '0,1%",IF(OR(NOT(ISTEXT(F29)),SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F29," ",""),"%",""),"'",""),".",",")="",ISERROR(_xlfn.NUMBERVALUE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F29," ",""),"%",""),"'",""),".",","),","," "))),"Ставка не распознана — наберите число, например 0,1 или 0,1%",IF(C29&lt;B29,"Окончание раньше начала — проверьте даты",IF(OR(E29&lt;0,_xlfn.NUMBERVALUE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F29," ",""),"%",""),"'",""),".",","),","," ")&lt;0),"База или ставка меньше нуля — проверьте ввод",IF(AND(_xlfn.NUMBERVALUE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F29," ",""),"%",""),"'",""),".",","),","," ")&gt;0,_xlfn.NUMBERVALUE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F29," ",""),"%",""),"'",""),".",","),","," ")&lt;1),"Ставка меньше 1 % годовых — книга такую ставку не считает",""))))))))</f>
         <v/>
       </c>
     </row>
@@ -909,13 +910,13 @@
         <v/>
       </c>
       <c r="E30" s="5" t="n"/>
-      <c r="F30" s="8" t="n"/>
-      <c r="G30" s="12">
-        <f>IF(OR(H30&lt;&gt;"",B30=""),"",E30*F30/100/365*D30)</f>
-        <v/>
-      </c>
-      <c r="H30" s="13">
-        <f>IF(AND(B30="",C30="",E30="",F30=""),"",IF(OR(B30="",C30="",E30="",F30=""),"Заполните все поля строки: начало, окончание, базу и ставку",IF(OR(NOT(ISNUMBER(B30)),NOT(ISNUMBER(C30)),NOT(ISNUMBER(E30)),NOT(ISNUMBER(F30))),"Даты и суммы вводятся числом, даты — ДД.ММ.ГГГГ",IF(C30&lt;B30,"Окончание раньше начала — проверьте даты",IF(OR(E30&lt;0,F30&lt;0),"База или ставка меньше нуля — проверьте ввод",IF(AND(F30&gt;0,F30&lt;1),"Ставка меньше 1 % годовых — так бывает, если набрать знак %. Введите число без знака %: 16 % — как 16",""))))))</f>
+      <c r="F30" s="12" t="n"/>
+      <c r="G30" s="13">
+        <f>IF(OR(H30&lt;&gt;"",B30=""),"",E30*_xlfn.NUMBERVALUE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F30," ",""),"%",""),"'",""),".",","),","," ")/100/365*D30)</f>
+        <v/>
+      </c>
+      <c r="H30" s="14">
+        <f>IF(AND(B30="",C30="",E30="",F30=""),"",IF(OR(B30="",C30="",E30="",F30=""),"Заполните все поля строки: начало, окончание, базу и ставку",IF(OR(NOT(ISNUMBER(B30)),NOT(ISNUMBER(C30)),NOT(ISNUMBER(E30))),"Даты и суммы вводятся числом, даты — ДД.ММ.ГГГГ",IF(ISNUMBER(F30),"Ставка вставлена числом — не видно, был ли знак %. Наберите её заново с апострофом впереди: '0,1 или '0,1%",IF(OR(NOT(ISTEXT(F30)),SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F30," ",""),"%",""),"'",""),".",",")="",ISERROR(_xlfn.NUMBERVALUE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F30," ",""),"%",""),"'",""),".",","),","," "))),"Ставка не распознана — наберите число, например 0,1 или 0,1%",IF(C30&lt;B30,"Окончание раньше начала — проверьте даты",IF(OR(E30&lt;0,_xlfn.NUMBERVALUE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F30," ",""),"%",""),"'",""),".",","),","," ")&lt;0),"База или ставка меньше нуля — проверьте ввод",IF(AND(_xlfn.NUMBERVALUE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F30," ",""),"%",""),"'",""),".",","),","," ")&gt;0,_xlfn.NUMBERVALUE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F30," ",""),"%",""),"'",""),".",","),","," ")&lt;1),"Ставка меньше 1 % годовых — книга такую ставку не считает",""))))))))</f>
         <v/>
       </c>
     </row>
@@ -930,13 +931,13 @@
         <v/>
       </c>
       <c r="E31" s="5" t="n"/>
-      <c r="F31" s="8" t="n"/>
-      <c r="G31" s="12">
-        <f>IF(OR(H31&lt;&gt;"",B31=""),"",E31*F31/100/365*D31)</f>
-        <v/>
-      </c>
-      <c r="H31" s="13">
-        <f>IF(AND(B31="",C31="",E31="",F31=""),"",IF(OR(B31="",C31="",E31="",F31=""),"Заполните все поля строки: начало, окончание, базу и ставку",IF(OR(NOT(ISNUMBER(B31)),NOT(ISNUMBER(C31)),NOT(ISNUMBER(E31)),NOT(ISNUMBER(F31))),"Даты и суммы вводятся числом, даты — ДД.ММ.ГГГГ",IF(C31&lt;B31,"Окончание раньше начала — проверьте даты",IF(OR(E31&lt;0,F31&lt;0),"База или ставка меньше нуля — проверьте ввод",IF(AND(F31&gt;0,F31&lt;1),"Ставка меньше 1 % годовых — так бывает, если набрать знак %. Введите число без знака %: 16 % — как 16",""))))))</f>
+      <c r="F31" s="12" t="n"/>
+      <c r="G31" s="13">
+        <f>IF(OR(H31&lt;&gt;"",B31=""),"",E31*_xlfn.NUMBERVALUE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F31," ",""),"%",""),"'",""),".",","),","," ")/100/365*D31)</f>
+        <v/>
+      </c>
+      <c r="H31" s="14">
+        <f>IF(AND(B31="",C31="",E31="",F31=""),"",IF(OR(B31="",C31="",E31="",F31=""),"Заполните все поля строки: начало, окончание, базу и ставку",IF(OR(NOT(ISNUMBER(B31)),NOT(ISNUMBER(C31)),NOT(ISNUMBER(E31))),"Даты и суммы вводятся числом, даты — ДД.ММ.ГГГГ",IF(ISNUMBER(F31),"Ставка вставлена числом — не видно, был ли знак %. Наберите её заново с апострофом впереди: '0,1 или '0,1%",IF(OR(NOT(ISTEXT(F31)),SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F31," ",""),"%",""),"'",""),".",",")="",ISERROR(_xlfn.NUMBERVALUE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F31," ",""),"%",""),"'",""),".",","),","," "))),"Ставка не распознана — наберите число, например 0,1 или 0,1%",IF(C31&lt;B31,"Окончание раньше начала — проверьте даты",IF(OR(E31&lt;0,_xlfn.NUMBERVALUE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F31," ",""),"%",""),"'",""),".",","),","," ")&lt;0),"База или ставка меньше нуля — проверьте ввод",IF(AND(_xlfn.NUMBERVALUE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F31," ",""),"%",""),"'",""),".",","),","," ")&gt;0,_xlfn.NUMBERVALUE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F31," ",""),"%",""),"'",""),".",","),","," ")&lt;1),"Ставка меньше 1 % годовых — книга такую ставку не считает",""))))))))</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
NSP P5: fix leap-year interest without print regression; native Excel 81 checks [skip deploy]
</commit_message>
<xml_diff>
--- a/products-storage/07-uderzhaniya-shtrafy-zachety/04-raschet-ubytkov.xlsx
+++ b/products-storage/07-uderzhaniya-shtrafy-zachety/04-raschet-ubytkov.xlsx
@@ -94,7 +94,7 @@
     <t>Итого пени, руб.</t>
   </si>
   <si>
-    <t>3. ПРОЦЕНТЫ ПО СТ. 395 ГК РФ: база × ключевая ставка / 100 / 365 × дни</t>
+    <t>3. ПРОЦЕНТЫ ПО СТ. 395 ГК РФ: фактические дни каждого года — 365 / 366</t>
   </si>
   <si>
     <t>Ключевая ставка, % годовых (16 или 16%)</t>
@@ -959,7 +959,7 @@
       <c r="E27" s="1"/>
       <c r="F27" s="8"/>
       <c r="G27" s="9" t="str">
-        <f>IF(OR(H27&lt;&gt;"",B27=""),"",E27*_xlfn.NUMBERVALUE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F27," ",""),"%",""),"'",""),".",","),","," ")/100/365*D27)</f>
+        <f>IF(OR(H27&lt;&gt;"",B27=""),"",E27*_xlfn.NUMBERVALUE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F27," ",""),"%",""),"'",""),".",","),","," ")/100*IF(YEAR(B27)=YEAR(C27),D27/(DATE(YEAR(B27)+1,1,1)-DATE(YEAR(B27),1,1)),(DATE(YEAR(B27)+1,1,1)-B27)/(DATE(YEAR(B27)+1,1,1)-DATE(YEAR(B27),1,1))+YEAR(C27)-YEAR(B27)-1+(C27-DATE(YEAR(C27),1,1)+1)/(DATE(YEAR(C27)+1,1,1)-DATE(YEAR(C27),1,1))))</f>
         <v/>
       </c>
       <c r="H27" s="10" t="str">
@@ -980,7 +980,7 @@
       <c r="E28" s="1"/>
       <c r="F28" s="8"/>
       <c r="G28" s="9" t="str">
-        <f>IF(OR(H28&lt;&gt;"",B28=""),"",E28*_xlfn.NUMBERVALUE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F28," ",""),"%",""),"'",""),".",","),","," ")/100/365*D28)</f>
+        <f>IF(OR(H28&lt;&gt;"",B28=""),"",E28*_xlfn.NUMBERVALUE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F28," ",""),"%",""),"'",""),".",","),","," ")/100*IF(YEAR(B28)=YEAR(C28),D28/(DATE(YEAR(B28)+1,1,1)-DATE(YEAR(B28),1,1)),(DATE(YEAR(B28)+1,1,1)-B28)/(DATE(YEAR(B28)+1,1,1)-DATE(YEAR(B28),1,1))+YEAR(C28)-YEAR(B28)-1+(C28-DATE(YEAR(C28),1,1)+1)/(DATE(YEAR(C28)+1,1,1)-DATE(YEAR(C28),1,1))))</f>
         <v/>
       </c>
       <c r="H28" s="10" t="str">
@@ -1001,7 +1001,7 @@
       <c r="E29" s="1"/>
       <c r="F29" s="8"/>
       <c r="G29" s="9" t="str">
-        <f>IF(OR(H29&lt;&gt;"",B29=""),"",E29*_xlfn.NUMBERVALUE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F29," ",""),"%",""),"'",""),".",","),","," ")/100/365*D29)</f>
+        <f>IF(OR(H29&lt;&gt;"",B29=""),"",E29*_xlfn.NUMBERVALUE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F29," ",""),"%",""),"'",""),".",","),","," ")/100*IF(YEAR(B29)=YEAR(C29),D29/(DATE(YEAR(B29)+1,1,1)-DATE(YEAR(B29),1,1)),(DATE(YEAR(B29)+1,1,1)-B29)/(DATE(YEAR(B29)+1,1,1)-DATE(YEAR(B29),1,1))+YEAR(C29)-YEAR(B29)-1+(C29-DATE(YEAR(C29),1,1)+1)/(DATE(YEAR(C29)+1,1,1)-DATE(YEAR(C29),1,1))))</f>
         <v/>
       </c>
       <c r="H29" s="10" t="str">
@@ -1022,7 +1022,7 @@
       <c r="E30" s="1"/>
       <c r="F30" s="8"/>
       <c r="G30" s="9" t="str">
-        <f>IF(OR(H30&lt;&gt;"",B30=""),"",E30*_xlfn.NUMBERVALUE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F30," ",""),"%",""),"'",""),".",","),","," ")/100/365*D30)</f>
+        <f>IF(OR(H30&lt;&gt;"",B30=""),"",E30*_xlfn.NUMBERVALUE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F30," ",""),"%",""),"'",""),".",","),","," ")/100*IF(YEAR(B30)=YEAR(C30),D30/(DATE(YEAR(B30)+1,1,1)-DATE(YEAR(B30),1,1)),(DATE(YEAR(B30)+1,1,1)-B30)/(DATE(YEAR(B30)+1,1,1)-DATE(YEAR(B30),1,1))+YEAR(C30)-YEAR(B30)-1+(C30-DATE(YEAR(C30),1,1)+1)/(DATE(YEAR(C30)+1,1,1)-DATE(YEAR(C30),1,1))))</f>
         <v/>
       </c>
       <c r="H30" s="10" t="str">
@@ -1043,7 +1043,7 @@
       <c r="E31" s="1"/>
       <c r="F31" s="8"/>
       <c r="G31" s="9" t="str">
-        <f>IF(OR(H31&lt;&gt;"",B31=""),"",E31*_xlfn.NUMBERVALUE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F31," ",""),"%",""),"'",""),".",","),","," ")/100/365*D31)</f>
+        <f>IF(OR(H31&lt;&gt;"",B31=""),"",E31*_xlfn.NUMBERVALUE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F31," ",""),"%",""),"'",""),".",","),","," ")/100*IF(YEAR(B31)=YEAR(C31),D31/(DATE(YEAR(B31)+1,1,1)-DATE(YEAR(B31),1,1)),(DATE(YEAR(B31)+1,1,1)-B31)/(DATE(YEAR(B31)+1,1,1)-DATE(YEAR(B31),1,1))+YEAR(C31)-YEAR(B31)-1+(C31-DATE(YEAR(C31),1,1)+1)/(DATE(YEAR(C31)+1,1,1)-DATE(YEAR(C31),1,1))))</f>
         <v/>
       </c>
       <c r="H31" s="10" t="str">

</xml_diff>